<commit_message>
New update for web
</commit_message>
<xml_diff>
--- a/assets/export.xlsx
+++ b/assets/export.xlsx
@@ -1,96 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sepan\Desktop\Programming\Flutter\shooka_flutter\assets\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B300FDF-7B71-478E-B373-1D937E97B1F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>ردیف</t>
-  </si>
-  <si>
-    <t>اسامی نصب</t>
-  </si>
-  <si>
-    <t>شماره اشتراک</t>
-  </si>
-  <si>
-    <t>شهر</t>
-  </si>
-  <si>
-    <t>تاریخ نصب</t>
-  </si>
-  <si>
-    <t>موبایل مشترک</t>
-  </si>
-  <si>
-    <t>توضیحات</t>
-  </si>
-  <si>
-    <t>اسامی نصاب</t>
-  </si>
-  <si>
-    <t>شماره قرارداد</t>
-  </si>
-  <si>
-    <t xml:space="preserve">آدرس </t>
-  </si>
-  <si>
-    <t>شماره سریال دستگاه</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
       <name val="B Nazanin"/>
       <charset val="178"/>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
-      <sz val="12"/>
       <name val="B Nazanin"/>
       <charset val="178"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -130,30 +76,89 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -448,79 +453,109 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="6.69921875" customWidth="1"/>
-    <col min="2" max="2" width="33.3984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="17.19921875" customWidth="1"/>
-    <col min="5" max="5" width="12.3984375" customWidth="1"/>
-    <col min="6" max="6" width="14.3984375" customWidth="1"/>
-    <col min="7" max="7" width="25.59765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="11.8984375" customWidth="1"/>
-    <col min="10" max="10" width="11.3984375" customWidth="1"/>
-    <col min="11" max="11" width="50.59765625" customWidth="1"/>
-    <col min="12" max="14" width="8.69921875" customWidth="1"/>
+    <col width="6.69921875" customWidth="1" min="1" max="1"/>
+    <col width="33.3984375" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="17.19921875" customWidth="1" min="3" max="4"/>
+    <col width="12.3984375" customWidth="1" min="5" max="5"/>
+    <col width="14.3984375" customWidth="1" min="6" max="6"/>
+    <col width="25.59765625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11.9" customWidth="1" min="10" max="10"/>
+    <col width="11.4" customWidth="1" min="11" max="11"/>
+    <col width="50.6" customWidth="1" min="12" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ردیف</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسامی نصب</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>شماره اشتراک</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>شهر</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تاریخ نصب</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>موبایل مشترک</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>شماره سریال دستگاه</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>کد داخلی دستگاه</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>توضیحات</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>اسامی نصاب</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>شماره قرارداد</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>آدرس</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
     </row>
-    <row r="2" spans="1:14" ht="18.75" customHeight="1">
-      <c r="A2" s="3"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" s="3" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape" r:id="rId1"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>